<commit_message>
1.测试新的onnx导出方案； 2. 增加onnx fp16导出； 3. 增加inceptionnext_tiny和inceptionnext_tiny_pro测试
</commit_message>
<xml_diff>
--- a/测试数据.xlsx
+++ b/测试数据.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\F\ABlueFaceProj\20240618\Seg\Beta_BiSeNet-master_Slim\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A68ABC9-8850-4D09-A165-62B3E3531163}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{965B487F-2EEB-4636-B4E4-76678BA29646}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="147">
   <si>
     <t>x2</t>
   </si>
@@ -459,6 +459,26 @@
   </si>
   <si>
     <t>prgseg_hgnetv2_b6</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>fastefficientbisenet_inceptionnext_atto</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.754584/0.760426</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.772044/0.777559</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>fastefficientbisenet_inceptionnext_tiny</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>fastefficientbisenet_inceptionnext_tiny_pro</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -539,7 +559,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -552,10 +572,25 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -831,1196 +866,1289 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O56"/>
+  <dimension ref="A1:M58"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="59.109375" customWidth="1"/>
-    <col min="2" max="2" width="15.109375" customWidth="1"/>
+    <col min="1" max="1" width="46.88671875" customWidth="1"/>
+    <col min="2" max="2" width="11.77734375" customWidth="1"/>
     <col min="3" max="3" width="10.88671875" customWidth="1"/>
     <col min="4" max="4" width="10.44140625" customWidth="1"/>
-    <col min="6" max="8" width="9.6640625"/>
-    <col min="9" max="9" width="11.44140625" customWidth="1"/>
-    <col min="10" max="11" width="9.6640625"/>
+    <col min="5" max="5" width="9.88671875" customWidth="1"/>
+    <col min="6" max="6" width="9.6640625"/>
+    <col min="7" max="7" width="22.44140625" customWidth="1"/>
+    <col min="8" max="8" width="9.6640625"/>
+    <col min="9" max="9" width="9.109375" customWidth="1"/>
+    <col min="11" max="11" width="17.88671875" customWidth="1"/>
     <col min="12" max="12" width="15.21875" customWidth="1"/>
-    <col min="13" max="13" width="13.44140625" customWidth="1"/>
-    <col min="14" max="14" width="22.33203125" customWidth="1"/>
+    <col min="13" max="13" width="12.33203125" customWidth="1"/>
+    <col min="14" max="14" width="18.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="E1" s="7" t="s">
         <v>140</v>
       </c>
-      <c r="I1" t="s">
+      <c r="F1" s="1">
+        <v>6</v>
+      </c>
+      <c r="G1" s="1">
+        <v>8</v>
+      </c>
+      <c r="H1" s="1">
+        <v>9</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="N1" s="9" t="s">
+      <c r="K1" s="6" t="s">
         <v>137</v>
       </c>
-      <c r="O1" s="9" t="s">
+      <c r="L1" s="6" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="M1" s="6"/>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="1">
         <v>0.77989699999999995</v>
       </c>
-      <c r="C2">
+      <c r="C2" s="1">
         <v>0.89335799999999999</v>
       </c>
-      <c r="D2">
+      <c r="D2" s="1">
         <v>0.85520099999999999</v>
       </c>
-      <c r="F2">
+      <c r="E2" s="1"/>
+      <c r="F2" s="1">
         <v>0.78461199999999998</v>
       </c>
-      <c r="G2">
-        <v>0.89091500000000001</v>
-      </c>
-      <c r="H2">
-        <v>0.86289400000000005</v>
-      </c>
-      <c r="I2" t="s">
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="1">
         <v>0.77761400000000003</v>
       </c>
-      <c r="C3">
+      <c r="C3" s="1">
         <v>0.88759200000000005</v>
       </c>
-      <c r="D3">
+      <c r="D3" s="1">
         <v>0.85787100000000005</v>
       </c>
-      <c r="F3">
+      <c r="E3" s="1"/>
+      <c r="F3" s="1">
         <v>0.79134499999999997</v>
       </c>
-      <c r="G3">
-        <v>0.89273899999999995</v>
-      </c>
-      <c r="H3">
-        <v>0.86963800000000002</v>
-      </c>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="G3" s="1"/>
+      <c r="H3" s="1"/>
+      <c r="I3" s="1"/>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="1">
         <v>0.77242900000000003</v>
       </c>
-      <c r="C4">
+      <c r="C4" s="1">
         <v>0.89129499999999995</v>
       </c>
-      <c r="D4">
+      <c r="D4" s="1">
         <v>0.84928499999999996</v>
       </c>
-      <c r="I4">
+      <c r="E4" s="1"/>
+      <c r="F4" s="1"/>
+      <c r="G4" s="1"/>
+      <c r="H4" s="1"/>
+      <c r="I4" s="1">
         <v>124</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A5" s="6" t="s">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A5" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="1">
         <v>0.770065</v>
       </c>
-      <c r="C5">
+      <c r="C5" s="1">
         <v>0.88427999999999995</v>
       </c>
-      <c r="D5">
+      <c r="D5" s="1">
         <v>0.85091300000000003</v>
       </c>
-      <c r="F5">
+      <c r="E5" s="1"/>
+      <c r="F5" s="1">
         <v>0.76847900000000002</v>
       </c>
-      <c r="G5">
-        <v>0.86373599999999995</v>
-      </c>
-      <c r="H5">
-        <v>0.86833300000000002</v>
-      </c>
-      <c r="I5">
+      <c r="G5" s="7" t="s">
+        <v>144</v>
+      </c>
+      <c r="H5" s="1">
+        <v>0.76789700000000005</v>
+      </c>
+      <c r="I5" s="1">
         <v>49</v>
       </c>
-      <c r="J5">
-        <v>0.77204399999999995</v>
-      </c>
       <c r="K5">
-        <v>0.88118799999999997</v>
-      </c>
-      <c r="L5">
-        <v>0.85651299999999997</v>
-      </c>
-      <c r="N5">
         <v>1.4411799999999999</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B6">
+      <c r="B6" s="1">
         <v>0.76773199999999997</v>
       </c>
-      <c r="C6">
+      <c r="C6" s="1">
         <v>0.87141900000000005</v>
       </c>
-      <c r="D6">
+      <c r="D6" s="1">
         <v>0.86139500000000002</v>
       </c>
-      <c r="F6">
+      <c r="E6" s="1"/>
+      <c r="F6" s="1">
         <v>0.77103999999999995</v>
       </c>
-      <c r="G6">
-        <v>0.86763100000000004</v>
-      </c>
-      <c r="H6">
-        <v>0.86818799999999996</v>
-      </c>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+      <c r="G6" s="1"/>
+      <c r="H6" s="1"/>
+      <c r="I6" s="1"/>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A7" s="12" t="s">
+        <v>141</v>
+      </c>
+      <c r="B7" s="1">
+        <v>0.766594</v>
+      </c>
+      <c r="C7" s="1">
+        <v>0.88039100000000003</v>
+      </c>
+      <c r="D7" s="1">
+        <v>0.84912100000000001</v>
+      </c>
+      <c r="E7" s="1"/>
+      <c r="F7" s="1"/>
+      <c r="G7" s="1">
+        <v>0.77905599999999997</v>
+      </c>
+      <c r="H7" s="1"/>
+      <c r="I7" s="1"/>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B7">
+      <c r="B8" s="1">
         <v>0.76629499999999995</v>
       </c>
-      <c r="C7">
+      <c r="C8" s="1">
         <v>0.88547200000000004</v>
       </c>
-      <c r="D7">
+      <c r="D8" s="1">
         <v>0.84465999999999997</v>
       </c>
-      <c r="F7">
+      <c r="E8" s="1"/>
+      <c r="F8" s="1">
         <v>0.77436899999999997</v>
       </c>
-      <c r="G7">
-        <v>0.89326300000000003</v>
-      </c>
-      <c r="H7">
-        <v>0.84846699999999997</v>
-      </c>
-      <c r="I7">
+      <c r="G8" s="1"/>
+      <c r="H8" s="1"/>
+      <c r="I8" s="1">
         <v>85.6</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B8">
+      <c r="B9" s="1">
         <v>0.76426000000000005</v>
       </c>
-      <c r="C8">
+      <c r="C9" s="1">
         <v>0.88559200000000005</v>
       </c>
-      <c r="D8">
+      <c r="D9" s="1">
         <v>0.84231500000000004</v>
       </c>
-      <c r="I8">
+      <c r="E9" s="1"/>
+      <c r="F9" s="1"/>
+      <c r="G9" s="1"/>
+      <c r="H9" s="1"/>
+      <c r="I9" s="1">
         <v>58.84</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B9">
+      <c r="B10" s="1">
         <v>0.76256900000000005</v>
       </c>
-      <c r="C9">
+      <c r="C10" s="1">
         <v>0.88412100000000005</v>
       </c>
-      <c r="D9">
+      <c r="D10" s="1">
         <v>0.84111400000000003</v>
       </c>
-      <c r="I9">
+      <c r="E10" s="1"/>
+      <c r="F10" s="1"/>
+      <c r="G10" s="1"/>
+      <c r="H10" s="1"/>
+      <c r="I10" s="1">
         <v>115</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B10">
+      <c r="B11" s="1">
         <v>0.76244999999999996</v>
       </c>
-      <c r="C10">
+      <c r="C11" s="1">
         <v>0.88131199999999998</v>
       </c>
-      <c r="D10">
+      <c r="D11" s="1">
         <v>0.84433000000000002</v>
       </c>
-      <c r="I10">
+      <c r="E11" s="1"/>
+      <c r="F11" s="1"/>
+      <c r="G11" s="1"/>
+      <c r="H11" s="1"/>
+      <c r="I11" s="1">
         <v>113</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B11">
+      <c r="B12" s="1">
         <v>0.76091900000000001</v>
       </c>
-      <c r="C11">
+      <c r="C12" s="1">
         <v>0.87430300000000005</v>
       </c>
-      <c r="D11">
+      <c r="D12" s="1">
         <v>0.84851699999999997</v>
       </c>
-    </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+      <c r="E12" s="1"/>
+      <c r="F12" s="1"/>
+      <c r="G12" s="1"/>
+      <c r="H12" s="1"/>
+      <c r="I12" s="1"/>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B12">
+      <c r="B13" s="1">
         <v>0.76035600000000003</v>
       </c>
-      <c r="C12">
+      <c r="C13" s="1">
         <v>0.88488699999999998</v>
       </c>
-      <c r="D12">
+      <c r="D13" s="1">
         <v>0.83660800000000002</v>
       </c>
-      <c r="F12">
+      <c r="E13" s="1"/>
+      <c r="F13" s="1">
         <v>0.76341099999999995</v>
       </c>
-      <c r="G12">
-        <v>0.89001699999999995</v>
-      </c>
-      <c r="H12">
-        <v>0.83723499999999995</v>
-      </c>
-    </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+      <c r="G13" s="1"/>
+      <c r="H13" s="1"/>
+      <c r="I13" s="1"/>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B13">
+      <c r="B14" s="1">
         <v>0.75666599999999995</v>
       </c>
-      <c r="C13">
+      <c r="C14" s="1">
         <v>0.88330500000000001</v>
       </c>
-      <c r="D13">
+      <c r="D14" s="1">
         <v>0.83460699999999999</v>
       </c>
-    </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+      <c r="E14" s="1"/>
+      <c r="F14" s="1"/>
+      <c r="G14" s="1"/>
+      <c r="H14" s="1"/>
+      <c r="I14" s="1"/>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B14">
+      <c r="B15" s="1">
         <v>0.75477700000000003</v>
       </c>
-      <c r="C14">
+      <c r="C15" s="1">
         <v>0.863089</v>
       </c>
-      <c r="D14">
+      <c r="D15" s="1">
         <v>0.85082599999999997</v>
       </c>
-    </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
+      <c r="E15" s="1"/>
+      <c r="F15" s="1"/>
+      <c r="G15" s="1"/>
+      <c r="H15" s="1"/>
+      <c r="I15" s="1"/>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B15">
+      <c r="B16" s="1">
         <v>0.75433399999999995</v>
       </c>
-      <c r="C15">
+      <c r="C16" s="1">
         <v>0.873749</v>
       </c>
-      <c r="D15">
+      <c r="D16" s="1">
         <v>0.84041299999999997</v>
       </c>
-      <c r="F15">
+      <c r="E16" s="1"/>
+      <c r="F16" s="1">
         <v>0.75883900000000004</v>
       </c>
-      <c r="G15">
-        <v>0.86963000000000001</v>
-      </c>
-      <c r="H15">
-        <v>0.84927200000000003</v>
-      </c>
-      <c r="I15">
+      <c r="G16" s="1"/>
+      <c r="H16" s="1"/>
+      <c r="I16" s="1">
         <v>69.849999999999994</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+    <row r="17" spans="1:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B16">
+      <c r="B17" s="1">
         <v>0.75273599999999996</v>
       </c>
-      <c r="C16">
+      <c r="C17" s="1">
         <v>0.88347399999999998</v>
       </c>
-      <c r="D16">
+      <c r="D17" s="1">
         <v>0.82959099999999997</v>
       </c>
-    </row>
-    <row r="17" spans="1:15" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="6" t="s">
+      <c r="E17" s="1"/>
+      <c r="F17" s="1"/>
+      <c r="G17" s="1"/>
+      <c r="H17" s="1"/>
+      <c r="I17" s="1"/>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A18" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="B17">
+      <c r="B18" s="1">
         <v>0.75112999999999996</v>
       </c>
-      <c r="C17">
+      <c r="C18" s="1">
         <v>0.88185500000000006</v>
       </c>
-      <c r="D17">
+      <c r="D18" s="1">
         <v>0.82863299999999995</v>
       </c>
-      <c r="F17">
+      <c r="E18" s="1"/>
+      <c r="F18" s="1">
         <v>0.75516300000000003</v>
       </c>
-      <c r="G17">
-        <v>0.87317900000000004</v>
-      </c>
-      <c r="H17">
-        <v>0.84089100000000006</v>
-      </c>
-      <c r="I17">
+      <c r="G18" s="1"/>
+      <c r="H18" s="1"/>
+      <c r="I18" s="1">
         <v>31.4</v>
       </c>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A18" s="6" t="s">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A19" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="B18">
+      <c r="B19" s="1">
         <v>0.74993100000000001</v>
       </c>
-      <c r="C18">
+      <c r="C19" s="1">
         <v>0.88971900000000004</v>
       </c>
-      <c r="D18">
+      <c r="D19" s="1">
         <v>0.82317799999999997</v>
       </c>
-      <c r="F18">
+      <c r="E19" s="1"/>
+      <c r="F19" s="1">
         <v>0.75429500000000005</v>
       </c>
-      <c r="G18">
-        <v>0.86771600000000004</v>
-      </c>
-      <c r="H18">
-        <v>0.84682100000000005</v>
-      </c>
-      <c r="I18">
+      <c r="G19" s="1">
+        <v>0.75837500000000002</v>
+      </c>
+      <c r="H19" s="1"/>
+      <c r="I19" s="1">
         <v>21.2</v>
       </c>
-      <c r="J18">
-        <v>0.75837500000000002</v>
-      </c>
-      <c r="K18">
-        <v>0.88571699999999998</v>
-      </c>
-      <c r="L18">
-        <v>0.83616599999999996</v>
-      </c>
-    </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A19" s="6" t="s">
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A20" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="B20" s="1">
+        <v>0.74903500000000001</v>
+      </c>
+      <c r="C20" s="1">
+        <v>0.86494899999999997</v>
+      </c>
+      <c r="D20" s="1">
+        <v>0.84147300000000003</v>
+      </c>
+      <c r="E20" s="1"/>
+      <c r="F20" s="1"/>
+      <c r="G20" s="1"/>
+      <c r="H20" s="1"/>
+      <c r="I20" s="1"/>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A21" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="B19">
+      <c r="B21" s="1">
         <v>0.74761</v>
       </c>
-      <c r="C19">
+      <c r="C21" s="1">
         <v>0.864012</v>
       </c>
-      <c r="D19">
+      <c r="D21" s="1">
         <v>0.84015300000000004</v>
       </c>
-      <c r="F19">
+      <c r="E21" s="1"/>
+      <c r="F21" s="1">
         <v>0.74314100000000005</v>
       </c>
-      <c r="G19">
-        <v>0.87060499999999996</v>
-      </c>
-      <c r="H19">
-        <v>0.82750800000000002</v>
-      </c>
-      <c r="I19">
+      <c r="G21" s="1"/>
+      <c r="H21" s="1"/>
+      <c r="I21" s="1">
         <v>37</v>
       </c>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A22" s="9" t="s">
+        <v>136</v>
+      </c>
+      <c r="B22" s="1">
+        <v>0.74725900000000001</v>
+      </c>
+      <c r="C22" s="1">
+        <v>0.86913899999999999</v>
+      </c>
+      <c r="D22" s="1">
+        <v>0.835422</v>
+      </c>
+      <c r="E22" s="1"/>
+      <c r="F22" s="1"/>
+      <c r="G22" s="1"/>
+      <c r="H22" s="1"/>
+      <c r="I22" s="1"/>
+      <c r="K22">
+        <v>3.6217100000000002</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B20">
+      <c r="B23" s="1">
         <v>0.74657700000000005</v>
       </c>
-      <c r="C20">
+      <c r="C23" s="1">
         <v>0.86698200000000003</v>
       </c>
-      <c r="D20">
+      <c r="D23" s="1">
         <v>0.836866</v>
       </c>
-    </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A21" s="6" t="s">
+      <c r="E23" s="1"/>
+      <c r="F23" s="1"/>
+      <c r="G23" s="1"/>
+      <c r="H23" s="1"/>
+      <c r="I23" s="1"/>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A24" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="B24" s="1">
+        <v>0.74578599999999995</v>
+      </c>
+      <c r="C24" s="1">
+        <v>0.87922</v>
+      </c>
+      <c r="D24" s="1">
+        <v>0.82449899999999998</v>
+      </c>
+      <c r="E24" s="1"/>
+      <c r="F24" s="1"/>
+      <c r="G24" s="1">
+        <v>0.74951400000000001</v>
+      </c>
+      <c r="H24" s="1"/>
+      <c r="I24" s="1"/>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A25" s="9" t="s">
+        <v>142</v>
+      </c>
+      <c r="B25" s="1">
+        <v>0.74468699999999999</v>
+      </c>
+      <c r="C25" s="1">
+        <v>0.88054699999999997</v>
+      </c>
+      <c r="D25" s="1">
+        <v>0.82219600000000004</v>
+      </c>
+      <c r="E25" s="1">
+        <v>0.75261500000000003</v>
+      </c>
+      <c r="F25" s="1">
+        <v>0.75131099999999995</v>
+      </c>
+      <c r="G25" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="H25" s="1">
+        <v>0.76078100000000004</v>
+      </c>
+      <c r="I25" s="1">
+        <v>14.5</v>
+      </c>
+      <c r="K25">
+        <v>0.75868000000000002</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A26" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B26" s="1">
+        <v>0.74462200000000001</v>
+      </c>
+      <c r="C26" s="1">
+        <v>0.87063699999999999</v>
+      </c>
+      <c r="D26" s="1">
+        <v>0.83057499999999995</v>
+      </c>
+      <c r="E26" s="1"/>
+      <c r="F26" s="1"/>
+      <c r="G26" s="1"/>
+      <c r="H26" s="1"/>
+      <c r="I26" s="1">
+        <v>88.3</v>
+      </c>
+      <c r="L26">
+        <v>0.88</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A27" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="B27" s="10">
+        <v>0.744506</v>
+      </c>
+      <c r="C27" s="10">
+        <v>0.86052799999999996</v>
+      </c>
+      <c r="D27" s="10">
+        <v>0.83985100000000001</v>
+      </c>
+      <c r="E27" s="10"/>
+      <c r="F27" s="10">
+        <v>0.75157399999999996</v>
+      </c>
+      <c r="G27" s="1"/>
+      <c r="H27" s="10"/>
+      <c r="I27" s="10">
+        <v>57.3</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A28" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B28" s="1">
+        <v>0.74432399999999999</v>
+      </c>
+      <c r="C28" s="1">
+        <v>0.88753000000000004</v>
+      </c>
+      <c r="D28" s="1">
+        <v>0.81701400000000002</v>
+      </c>
+      <c r="E28" s="1"/>
+      <c r="F28" s="1"/>
+      <c r="G28" s="1"/>
+      <c r="H28" s="1"/>
+      <c r="I28" s="1"/>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A29" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B29" s="1">
+        <v>0.743591</v>
+      </c>
+      <c r="C29" s="1">
+        <v>0.872448</v>
+      </c>
+      <c r="D29" s="1">
+        <v>0.82741100000000001</v>
+      </c>
+      <c r="E29" s="1"/>
+      <c r="F29" s="1"/>
+      <c r="G29" s="1"/>
+      <c r="H29" s="1"/>
+      <c r="I29" s="1"/>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A30" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="B30" s="1">
+        <v>0.74173299999999998</v>
+      </c>
+      <c r="C30" s="1">
+        <v>0.86497599999999997</v>
+      </c>
+      <c r="D30" s="1">
+        <v>0.83116299999999999</v>
+      </c>
+      <c r="E30" s="1"/>
+      <c r="F30" s="1">
+        <v>0.745726</v>
+      </c>
+      <c r="G30" s="1">
+        <v>0.75325799999999998</v>
+      </c>
+      <c r="H30" s="1"/>
+      <c r="I30" s="1">
+        <v>30.7</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A31" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B31" s="1">
+        <v>0.74162899999999998</v>
+      </c>
+      <c r="C31" s="1">
+        <v>0.86836000000000002</v>
+      </c>
+      <c r="D31" s="1">
+        <v>0.82718199999999997</v>
+      </c>
+      <c r="E31" s="1"/>
+      <c r="F31" s="1"/>
+      <c r="G31" s="1"/>
+      <c r="H31" s="1"/>
+      <c r="I31" s="1"/>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A32" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B32" s="1">
+        <v>0.740506</v>
+      </c>
+      <c r="C32" s="1">
+        <v>0.865591</v>
+      </c>
+      <c r="D32" s="1">
+        <v>0.82916100000000004</v>
+      </c>
+      <c r="E32" s="1"/>
+      <c r="F32" s="1">
+        <v>0.75195400000000001</v>
+      </c>
+      <c r="G32" s="1"/>
+      <c r="H32" s="1"/>
+      <c r="I32" s="1">
+        <v>50.5</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A33" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B33" s="1">
+        <v>0.73980500000000005</v>
+      </c>
+      <c r="C33" s="1">
+        <v>0.86816499999999996</v>
+      </c>
+      <c r="D33" s="1">
+        <v>0.82677999999999996</v>
+      </c>
+      <c r="E33" s="1"/>
+      <c r="F33" s="1"/>
+      <c r="G33" s="1"/>
+      <c r="H33" s="1"/>
+      <c r="I33" s="1"/>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A34" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B34" s="1">
+        <v>0.73975500000000005</v>
+      </c>
+      <c r="C34" s="1">
+        <v>0.85670999999999997</v>
+      </c>
+      <c r="D34" s="1">
+        <v>0.83675999999999995</v>
+      </c>
+      <c r="E34" s="1">
+        <v>0.74752300000000005</v>
+      </c>
+      <c r="F34" s="1"/>
+      <c r="G34" s="1">
+        <v>0.74913600000000002</v>
+      </c>
+      <c r="H34" s="1">
+        <v>0.75407299999999999</v>
+      </c>
+      <c r="I34" s="1">
+        <v>17.97</v>
+      </c>
+      <c r="K34">
+        <v>0.92</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A35" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="B35" s="1">
+        <v>0.73849100000000001</v>
+      </c>
+      <c r="C35" s="1">
+        <v>0.86501799999999995</v>
+      </c>
+      <c r="D35" s="1">
+        <v>0.827704</v>
+      </c>
+      <c r="E35" s="1"/>
+      <c r="F35" s="1">
+        <v>0.74363000000000001</v>
+      </c>
+      <c r="G35" s="1"/>
+      <c r="H35" s="1"/>
+      <c r="I35" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A36" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B36" s="1">
+        <v>0.73821400000000004</v>
+      </c>
+      <c r="C36" s="1">
+        <v>0.86428000000000005</v>
+      </c>
+      <c r="D36" s="1">
+        <v>0.82671399999999995</v>
+      </c>
+      <c r="E36" s="1"/>
+      <c r="F36" s="1"/>
+      <c r="G36" s="1"/>
+      <c r="H36" s="1"/>
+      <c r="I36" s="1"/>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A37" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B37" s="1">
+        <v>0.73571799999999998</v>
+      </c>
+      <c r="C37" s="1">
+        <v>0.87732399999999999</v>
+      </c>
+      <c r="D37" s="1">
+        <v>0.81230599999999997</v>
+      </c>
+      <c r="E37" s="1"/>
+      <c r="F37" s="1"/>
+      <c r="G37" s="1"/>
+      <c r="H37" s="1"/>
+      <c r="I37" s="1">
+        <v>16.73</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A38" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="B38" s="1">
+        <v>0.73497599999999996</v>
+      </c>
+      <c r="C38" s="1">
+        <v>0.86321599999999998</v>
+      </c>
+      <c r="D38" s="1">
+        <v>0.82403800000000005</v>
+      </c>
+      <c r="E38" s="1"/>
+      <c r="F38" s="1"/>
+      <c r="G38" s="1">
+        <v>0.74550499999999997</v>
+      </c>
+      <c r="H38" s="1"/>
+      <c r="I38" s="1">
+        <v>22.9</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A39" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="B39" s="1">
+        <v>0.73430099999999998</v>
+      </c>
+      <c r="C39" s="1">
+        <v>0.87199099999999996</v>
+      </c>
+      <c r="D39" s="1">
+        <v>0.81632199999999999</v>
+      </c>
+      <c r="E39" s="1"/>
+      <c r="F39" s="1"/>
+      <c r="G39" s="1">
+        <v>0.75073900000000005</v>
+      </c>
+      <c r="H39" s="1"/>
+      <c r="I39" s="1">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A40" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B40" s="1">
+        <v>0.73252300000000004</v>
+      </c>
+      <c r="C40" s="1">
+        <v>0.86758900000000005</v>
+      </c>
+      <c r="D40" s="1">
+        <v>0.81816699999999998</v>
+      </c>
+      <c r="E40" s="1"/>
+      <c r="F40" s="1"/>
+      <c r="G40" s="1"/>
+      <c r="H40" s="1"/>
+      <c r="I40" s="1"/>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A41" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B41" s="1">
+        <v>0.73216400000000004</v>
+      </c>
+      <c r="C41" s="1">
+        <v>0.86068100000000003</v>
+      </c>
+      <c r="D41" s="1">
+        <v>0.82388899999999998</v>
+      </c>
+      <c r="E41" s="1"/>
+      <c r="F41" s="1"/>
+      <c r="G41" s="1"/>
+      <c r="H41" s="1"/>
+      <c r="I41" s="1"/>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A42" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B42" s="1">
+        <v>0.73082899999999995</v>
+      </c>
+      <c r="C42" s="1">
+        <v>0.86943099999999995</v>
+      </c>
+      <c r="D42" s="1">
+        <v>0.81454800000000005</v>
+      </c>
+      <c r="E42" s="1"/>
+      <c r="F42" s="1"/>
+      <c r="G42" s="1"/>
+      <c r="H42" s="1"/>
+      <c r="I42" s="1"/>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A43" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B43" s="1">
+        <v>0.72680400000000001</v>
+      </c>
+      <c r="C43" s="1">
+        <v>0.857101</v>
+      </c>
+      <c r="D43" s="1">
+        <v>0.81938500000000003</v>
+      </c>
+      <c r="E43" s="1"/>
+      <c r="F43" s="1"/>
+      <c r="G43" s="1"/>
+      <c r="H43" s="1"/>
+      <c r="I43" s="1">
         <v>25</v>
       </c>
-      <c r="B21">
-        <v>0.74468699999999999</v>
-      </c>
-      <c r="C21">
-        <v>0.88054699999999997</v>
-      </c>
-      <c r="D21">
-        <v>0.82219600000000004</v>
-      </c>
-      <c r="E21">
-        <v>0.75261500000000003</v>
-      </c>
-      <c r="F21">
-        <v>0.75131099999999995</v>
-      </c>
-      <c r="G21">
-        <v>0.88209899999999997</v>
-      </c>
-      <c r="H21">
-        <v>0.83011900000000005</v>
-      </c>
-      <c r="I21">
-        <v>14.5</v>
-      </c>
-      <c r="J21">
-        <v>0.75458400000000003</v>
-      </c>
-      <c r="K21">
-        <v>0.87913799999999998</v>
-      </c>
-      <c r="L21">
-        <v>0.836511</v>
-      </c>
-      <c r="N21">
-        <v>0.75868000000000002</v>
-      </c>
-      <c r="O21">
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A44" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B44" s="1">
+        <v>0.72399400000000003</v>
+      </c>
+      <c r="C44" s="1">
+        <v>0.85761799999999999</v>
+      </c>
+      <c r="D44" s="1">
+        <v>0.81521999999999994</v>
+      </c>
+      <c r="E44" s="1"/>
+      <c r="F44" s="1"/>
+      <c r="G44" s="1"/>
+      <c r="H44" s="1"/>
+      <c r="I44" s="1"/>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A45" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="B45" s="1">
+        <v>0.72123300000000001</v>
+      </c>
+      <c r="C45" s="1">
+        <v>0.85792599999999997</v>
+      </c>
+      <c r="D45" s="1">
+        <v>0.81019799999999997</v>
+      </c>
+      <c r="E45" s="1"/>
+      <c r="F45" s="1"/>
+      <c r="G45" s="1">
+        <v>0.73479399999999995</v>
+      </c>
+      <c r="H45" s="1"/>
+      <c r="I45" s="1">
+        <v>11.42</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A46" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B46" s="1">
+        <v>0.71946500000000002</v>
+      </c>
+      <c r="C46" s="1">
+        <v>0.86807000000000001</v>
+      </c>
+      <c r="D46" s="1">
+        <v>0.80044899999999997</v>
+      </c>
+      <c r="E46" s="1"/>
+      <c r="F46" s="1"/>
+      <c r="G46" s="1"/>
+      <c r="H46" s="1"/>
+      <c r="I46" s="1"/>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A47" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B47" s="1">
+        <v>0.71696099999999996</v>
+      </c>
+      <c r="C47" s="1">
+        <v>0.870251</v>
+      </c>
+      <c r="D47" s="1">
+        <v>0.79447199999999996</v>
+      </c>
+      <c r="E47" s="1"/>
+      <c r="F47" s="1"/>
+      <c r="G47" s="1"/>
+      <c r="H47" s="1"/>
+      <c r="I47" s="1">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A48" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B48" s="1">
+        <v>0.71694000000000002</v>
+      </c>
+      <c r="C48" s="1">
+        <v>0.86188799999999999</v>
+      </c>
+      <c r="D48" s="1">
+        <v>0.80137999999999998</v>
+      </c>
+      <c r="E48" s="1"/>
+      <c r="F48" s="1"/>
+      <c r="G48" s="1"/>
+      <c r="H48" s="1"/>
+      <c r="I48" s="1"/>
+    </row>
+    <row r="49" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A49" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="B49" s="1">
+        <v>0.71636500000000003</v>
+      </c>
+      <c r="C49" s="1">
+        <v>0.85087000000000002</v>
+      </c>
+      <c r="D49" s="1">
+        <v>0.81111999999999995</v>
+      </c>
+      <c r="E49" s="1"/>
+      <c r="F49" s="1"/>
+      <c r="G49" s="1">
+        <v>0.73605299999999996</v>
+      </c>
+      <c r="H49" s="1"/>
+      <c r="I49" s="1">
+        <v>7.71</v>
+      </c>
+    </row>
+    <row r="50" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A50" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B50" s="1">
+        <v>0.71354600000000001</v>
+      </c>
+      <c r="C50" s="1">
+        <v>0.869784</v>
+      </c>
+      <c r="D50" s="1">
+        <v>0.79198400000000002</v>
+      </c>
+      <c r="E50" s="1"/>
+      <c r="F50" s="1"/>
+      <c r="G50" s="1"/>
+      <c r="H50" s="1"/>
+      <c r="I50" s="1"/>
+    </row>
+    <row r="51" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A51" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B51" s="1">
+        <v>0.71179099999999995</v>
+      </c>
+      <c r="C51" s="1">
+        <v>0.86646400000000001</v>
+      </c>
+      <c r="D51" s="1">
+        <v>0.79112199999999999</v>
+      </c>
+      <c r="E51" s="1"/>
+      <c r="F51" s="1"/>
+      <c r="G51" s="1"/>
+      <c r="H51" s="1"/>
+      <c r="I51" s="1"/>
+    </row>
+    <row r="52" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A52" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B52" s="1">
+        <v>0.711113</v>
+      </c>
+      <c r="C52" s="1">
+        <v>0.84625399999999995</v>
+      </c>
+      <c r="D52" s="1">
+        <v>0.806975</v>
+      </c>
+      <c r="E52" s="1"/>
+      <c r="F52" s="1"/>
+      <c r="G52" s="1"/>
+      <c r="H52" s="1"/>
+      <c r="I52" s="1"/>
+    </row>
+    <row r="53" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A53" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="B53" s="1">
+        <v>0.71059899999999998</v>
+      </c>
+      <c r="C53" s="1">
+        <v>0.86808399999999997</v>
+      </c>
+      <c r="D53" s="1">
+        <v>0.78952599999999995</v>
+      </c>
+      <c r="E53" s="1"/>
+      <c r="F53" s="1"/>
+      <c r="G53" s="1">
+        <v>0.71683799999999998</v>
+      </c>
+      <c r="H53" s="1"/>
+      <c r="I53" s="1">
+        <v>25</v>
+      </c>
+      <c r="L53">
         <v>0.35229700000000003</v>
       </c>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A22" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="B22">
-        <v>0.74462200000000001</v>
-      </c>
-      <c r="C22">
-        <v>0.87063699999999999</v>
-      </c>
-      <c r="D22">
-        <v>0.83057499999999995</v>
-      </c>
-      <c r="I22">
-        <v>88.3</v>
-      </c>
-    </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A23" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="B23" s="4">
-        <v>0.744506</v>
-      </c>
-      <c r="C23" s="4">
-        <v>0.86052799999999996</v>
-      </c>
-      <c r="D23" s="4">
-        <v>0.83985100000000001</v>
-      </c>
-      <c r="E23" s="4"/>
-      <c r="F23" s="4">
-        <v>0.75157399999999996</v>
-      </c>
-      <c r="G23" s="4">
-        <v>0.86825699999999995</v>
-      </c>
-      <c r="H23" s="4">
-        <v>0.84174099999999996</v>
-      </c>
-      <c r="I23" s="4">
-        <v>57.3</v>
-      </c>
-    </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>28</v>
-      </c>
-      <c r="B24">
-        <v>0.74432399999999999</v>
-      </c>
-      <c r="C24">
-        <v>0.88753000000000004</v>
-      </c>
-      <c r="D24">
-        <v>0.81701400000000002</v>
-      </c>
-    </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>29</v>
-      </c>
-      <c r="B25">
-        <v>0.743591</v>
-      </c>
-      <c r="C25">
-        <v>0.872448</v>
-      </c>
-      <c r="D25">
-        <v>0.82741100000000001</v>
-      </c>
-    </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A26" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="B26">
-        <v>0.74173299999999998</v>
-      </c>
-      <c r="C26">
-        <v>0.86497599999999997</v>
-      </c>
-      <c r="D26">
-        <v>0.83116299999999999</v>
-      </c>
-      <c r="F26">
-        <v>0.745726</v>
-      </c>
-      <c r="G26">
-        <v>0.85971900000000001</v>
-      </c>
-      <c r="H26">
-        <v>0.84069199999999999</v>
-      </c>
-      <c r="I26">
-        <v>30.7</v>
-      </c>
-      <c r="J26">
-        <v>0.75325799999999998</v>
-      </c>
-      <c r="K26">
-        <v>0.86073</v>
-      </c>
-      <c r="L26">
-        <v>0.85052700000000003</v>
-      </c>
-    </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>31</v>
-      </c>
-      <c r="B27">
-        <v>0.74162899999999998</v>
-      </c>
-      <c r="C27">
-        <v>0.86836000000000002</v>
-      </c>
-      <c r="D27">
-        <v>0.82718199999999997</v>
-      </c>
-    </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>32</v>
-      </c>
-      <c r="B28">
-        <v>0.740506</v>
-      </c>
-      <c r="C28">
-        <v>0.865591</v>
-      </c>
-      <c r="D28">
-        <v>0.82916100000000004</v>
-      </c>
-      <c r="F28">
-        <v>0.75195400000000001</v>
-      </c>
-      <c r="G28">
-        <v>0.86931199999999997</v>
-      </c>
-      <c r="H28">
-        <v>0.84161600000000003</v>
-      </c>
-      <c r="I28">
-        <v>50.5</v>
-      </c>
-    </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>33</v>
-      </c>
-      <c r="B29">
-        <v>0.73980500000000005</v>
-      </c>
-      <c r="C29">
-        <v>0.86816499999999996</v>
-      </c>
-      <c r="D29">
-        <v>0.82677999999999996</v>
-      </c>
-    </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A30" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="B30">
-        <v>0.73975500000000005</v>
-      </c>
-      <c r="C30">
-        <v>0.85670999999999997</v>
-      </c>
-      <c r="D30">
-        <v>0.83675999999999995</v>
-      </c>
-      <c r="I30">
-        <v>17.97</v>
-      </c>
-      <c r="J30">
-        <v>0.74913600000000002</v>
-      </c>
-      <c r="K30">
-        <v>0.85268299999999997</v>
-      </c>
-      <c r="L30">
-        <v>0.85444900000000001</v>
-      </c>
-    </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A31" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="B31">
-        <v>0.73849100000000001</v>
-      </c>
-      <c r="C31">
-        <v>0.86501799999999995</v>
-      </c>
-      <c r="D31">
-        <v>0.827704</v>
-      </c>
-      <c r="F31">
-        <v>0.74363000000000001</v>
-      </c>
-      <c r="G31">
-        <v>0.85514400000000002</v>
-      </c>
-      <c r="H31">
-        <v>0.84365900000000005</v>
-      </c>
-      <c r="I31" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="M31">
-        <v>30.6</v>
-      </c>
-    </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>37</v>
-      </c>
-      <c r="B32">
-        <v>0.73821400000000004</v>
-      </c>
-      <c r="C32">
-        <v>0.86428000000000005</v>
-      </c>
-      <c r="D32">
-        <v>0.82671399999999995</v>
-      </c>
-    </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>38</v>
-      </c>
-      <c r="B33">
-        <v>0.73571799999999998</v>
-      </c>
-      <c r="C33">
-        <v>0.87732399999999999</v>
-      </c>
-      <c r="D33">
-        <v>0.81230599999999997</v>
-      </c>
-      <c r="I33">
-        <v>16.73</v>
-      </c>
-    </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A34" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="B34">
-        <v>0.73430099999999998</v>
-      </c>
-      <c r="C34">
-        <v>0.87199099999999996</v>
-      </c>
-      <c r="D34">
-        <v>0.81632199999999999</v>
-      </c>
-      <c r="I34">
-        <v>31</v>
-      </c>
-      <c r="J34">
-        <v>0.75073900000000005</v>
-      </c>
-      <c r="K34">
-        <v>0.87304700000000002</v>
-      </c>
-      <c r="L34">
-        <v>0.83609699999999998</v>
-      </c>
-    </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>40</v>
-      </c>
-      <c r="B35">
-        <v>0.73252300000000004</v>
-      </c>
-      <c r="C35">
-        <v>0.86758900000000005</v>
-      </c>
-      <c r="D35">
-        <v>0.81816699999999998</v>
-      </c>
-    </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>41</v>
-      </c>
-      <c r="B36">
-        <v>0.73216400000000004</v>
-      </c>
-      <c r="C36">
-        <v>0.86068100000000003</v>
-      </c>
-      <c r="D36">
-        <v>0.82388899999999998</v>
-      </c>
-    </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>42</v>
-      </c>
-      <c r="B37">
-        <v>0.73082899999999995</v>
-      </c>
-      <c r="C37">
-        <v>0.86943099999999995</v>
-      </c>
-      <c r="D37">
-        <v>0.81454800000000005</v>
-      </c>
-    </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>43</v>
-      </c>
-      <c r="B38">
-        <v>0.72680400000000001</v>
-      </c>
-      <c r="C38">
-        <v>0.857101</v>
-      </c>
-      <c r="D38">
-        <v>0.81938500000000003</v>
-      </c>
-      <c r="I38">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
-        <v>44</v>
-      </c>
-      <c r="B39">
-        <v>0.72399400000000003</v>
-      </c>
-      <c r="C39">
-        <v>0.85761799999999999</v>
-      </c>
-      <c r="D39">
-        <v>0.81521999999999994</v>
-      </c>
-    </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
-        <v>45</v>
-      </c>
-      <c r="B40">
-        <v>0.71946500000000002</v>
-      </c>
-      <c r="C40">
-        <v>0.86807000000000001</v>
-      </c>
-      <c r="D40">
-        <v>0.80044899999999997</v>
-      </c>
-    </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
-        <v>46</v>
-      </c>
-      <c r="B41">
-        <v>0.71696099999999996</v>
-      </c>
-      <c r="C41">
-        <v>0.870251</v>
-      </c>
-      <c r="D41">
-        <v>0.79447199999999996</v>
-      </c>
-      <c r="I41">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
-        <v>47</v>
-      </c>
-      <c r="B42">
-        <v>0.71694000000000002</v>
-      </c>
-      <c r="C42">
-        <v>0.86188799999999999</v>
-      </c>
-      <c r="D42">
-        <v>0.80137999999999998</v>
-      </c>
-    </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A43" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="B43">
-        <v>0.71636500000000003</v>
-      </c>
-      <c r="C43">
-        <v>0.85087000000000002</v>
-      </c>
-      <c r="D43">
-        <v>0.81111999999999995</v>
-      </c>
-      <c r="I43">
-        <v>7.71</v>
-      </c>
-      <c r="J43">
-        <v>0.73605299999999996</v>
-      </c>
-      <c r="K43">
-        <v>0.85793399999999997</v>
-      </c>
-      <c r="L43">
-        <v>0.83193700000000004</v>
-      </c>
-    </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
-        <v>49</v>
-      </c>
-      <c r="B44">
-        <v>0.71354600000000001</v>
-      </c>
-      <c r="C44">
-        <v>0.869784</v>
-      </c>
-      <c r="D44">
-        <v>0.79198400000000002</v>
-      </c>
-    </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
-        <v>50</v>
-      </c>
-      <c r="B45">
-        <v>0.71179099999999995</v>
-      </c>
-      <c r="C45">
-        <v>0.86646400000000001</v>
-      </c>
-      <c r="D45">
-        <v>0.79112199999999999</v>
-      </c>
-    </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
-        <v>51</v>
-      </c>
-      <c r="B46">
-        <v>0.711113</v>
-      </c>
-      <c r="C46">
-        <v>0.84625399999999995</v>
-      </c>
-      <c r="D46">
-        <v>0.806975</v>
-      </c>
-    </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A47" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B47">
-        <v>0.71059899999999998</v>
-      </c>
-      <c r="C47">
-        <v>0.86808399999999997</v>
-      </c>
-      <c r="D47">
-        <v>0.78952599999999995</v>
-      </c>
-      <c r="I47">
-        <v>25</v>
-      </c>
-      <c r="J47">
-        <v>0.71683799999999998</v>
-      </c>
-      <c r="K47">
-        <v>0.848993</v>
-      </c>
-      <c r="L47">
-        <v>0.81343399999999999</v>
-      </c>
-    </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A48" s="6" t="s">
+    <row r="54" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A54" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="B48">
+      <c r="B54" s="1">
         <v>0.69976499999999997</v>
       </c>
-      <c r="C48">
+      <c r="C54" s="1">
         <v>0.84911899999999996</v>
       </c>
-      <c r="D48">
+      <c r="D54" s="1">
         <v>0.788358</v>
       </c>
-      <c r="F48">
+      <c r="E54" s="1"/>
+      <c r="F54" s="1">
         <v>0.69891499999999995</v>
       </c>
-      <c r="G48">
-        <v>0.847132</v>
-      </c>
-      <c r="H48">
-        <v>0.78894299999999995</v>
-      </c>
-      <c r="I48">
+      <c r="G54" s="1">
+        <v>0.71306599999999998</v>
+      </c>
+      <c r="H54" s="1"/>
+      <c r="I54" s="1">
         <v>9.74</v>
       </c>
-      <c r="J48">
-        <v>0.71306599999999998</v>
-      </c>
-      <c r="K48">
-        <v>0.852715</v>
-      </c>
-      <c r="L48">
-        <v>0.80514799999999997</v>
-      </c>
-    </row>
-    <row r="49" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A49" s="6" t="s">
+    </row>
+    <row r="55" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A55" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="B49">
+      <c r="B55" s="1">
         <v>0.69904900000000003</v>
       </c>
-      <c r="C49">
+      <c r="C55" s="1">
         <v>0.85933199999999998</v>
       </c>
-      <c r="D49">
+      <c r="D55" s="1">
         <v>0.781447</v>
       </c>
-      <c r="I49">
+      <c r="E55" s="1"/>
+      <c r="F55" s="1"/>
+      <c r="G55" s="1">
+        <v>0.69198599999999999</v>
+      </c>
+      <c r="H55" s="1"/>
+      <c r="I55" s="1">
         <v>12.94</v>
       </c>
-      <c r="J49">
-        <v>0.69198599999999999</v>
-      </c>
-      <c r="K49">
-        <v>0.83943800000000002</v>
-      </c>
-      <c r="L49">
-        <v>0.78869900000000004</v>
-      </c>
-    </row>
-    <row r="50" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
+    </row>
+    <row r="56" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A56" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="B50">
+      <c r="B56" s="1">
         <v>0.69497900000000001</v>
       </c>
-      <c r="C50">
+      <c r="C56" s="1">
         <v>0.86561600000000005</v>
       </c>
-      <c r="D50">
+      <c r="D56" s="1">
         <v>0.77168300000000001</v>
       </c>
-      <c r="F50">
+      <c r="E56" s="1"/>
+      <c r="F56" s="1">
         <v>0.69739899999999999</v>
       </c>
-      <c r="G50">
-        <v>0.868533</v>
-      </c>
-      <c r="H50">
-        <v>0.771671</v>
-      </c>
-    </row>
-    <row r="51" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A51" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="B51">
-        <v>0.73497599999999996</v>
-      </c>
-      <c r="C51">
-        <v>0.86321599999999998</v>
-      </c>
-      <c r="D51">
-        <v>0.82403800000000005</v>
-      </c>
-      <c r="I51">
-        <v>22.9</v>
-      </c>
-      <c r="J51">
-        <v>0.74550499999999997</v>
-      </c>
-      <c r="K51">
-        <v>0.86067899999999997</v>
-      </c>
-      <c r="L51">
-        <v>0.84021999999999997</v>
-      </c>
-    </row>
-    <row r="52" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A52" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="B52">
-        <v>0.72123300000000001</v>
-      </c>
-      <c r="C52">
-        <v>0.85792599999999997</v>
-      </c>
-      <c r="D52">
-        <v>0.81019799999999997</v>
-      </c>
-      <c r="I52">
-        <v>11.42</v>
-      </c>
-      <c r="J52">
-        <v>0.73479399999999995</v>
-      </c>
-      <c r="K52">
-        <v>0.85729500000000003</v>
-      </c>
-      <c r="L52">
-        <v>0.83084400000000003</v>
-      </c>
-    </row>
-    <row r="53" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A53" s="8" t="s">
-        <v>135</v>
-      </c>
-      <c r="B53">
-        <v>0.74578599999999995</v>
-      </c>
-      <c r="C53">
-        <v>0.87922</v>
-      </c>
-      <c r="D53">
-        <v>0.82449899999999998</v>
-      </c>
-      <c r="J53">
-        <v>0.74951400000000001</v>
-      </c>
-      <c r="K53">
-        <v>0.88462300000000005</v>
-      </c>
-      <c r="L53">
-        <v>0.82542499999999996</v>
-      </c>
-    </row>
-    <row r="54" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A54" s="8" t="s">
-        <v>136</v>
-      </c>
-      <c r="B54">
-        <v>0.74725900000000001</v>
-      </c>
-      <c r="C54">
-        <v>0.86913899999999999</v>
-      </c>
-      <c r="D54">
-        <v>0.835422</v>
-      </c>
-      <c r="N54">
-        <v>3.6217100000000002</v>
-      </c>
-    </row>
-    <row r="55" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A55" s="9" t="s">
-        <v>139</v>
-      </c>
-      <c r="B55">
-        <v>0.74903500000000001</v>
-      </c>
-      <c r="C55">
-        <v>0.86494899999999997</v>
-      </c>
-      <c r="D55">
-        <v>0.84147300000000003</v>
-      </c>
-    </row>
-    <row r="56" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A56" s="8" t="s">
-        <v>141</v>
-      </c>
-      <c r="B56">
-        <v>0.766594</v>
-      </c>
-      <c r="C56">
-        <v>0.88039100000000003</v>
-      </c>
-      <c r="D56">
-        <v>0.84912100000000001</v>
+      <c r="G56" s="1"/>
+      <c r="H56" s="1"/>
+      <c r="I56" s="1"/>
+    </row>
+    <row r="57" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A57" s="9" t="s">
+        <v>145</v>
+      </c>
+      <c r="B57" s="1">
+        <v>0.78243600000000002</v>
+      </c>
+      <c r="C57" s="1">
+        <v>0.89274200000000004</v>
+      </c>
+      <c r="D57" s="1">
+        <v>0.85849200000000003</v>
+      </c>
+      <c r="G57" s="1">
+        <v>0.78455699999999995</v>
+      </c>
+    </row>
+    <row r="58" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A58" s="9" t="s">
+        <v>146</v>
+      </c>
+      <c r="B58" s="1">
+        <v>0.78566499999999995</v>
+      </c>
+      <c r="C58" s="1">
+        <v>0.89692000000000005</v>
+      </c>
+      <c r="D58" s="1">
+        <v>0.85882999999999998</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:L50">
-    <sortCondition descending="1" ref="B1:B50"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L58">
+    <sortCondition descending="1" ref="B2:B58"/>
   </sortState>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>